<commit_message>
Ajoute la catégorie Gewestplan manquante "lokaal bedrijventerrein met openbaar karakter"
Même correctif que cloud/ (voir ce dépôt pour le détail complet et les
vérifications). Gabarit, colonnes_be.py et resolveur_service.py mis à
jour et vérifiés identiques entre les deux dépôts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/gabarit_officiel.xlsx
+++ b/templates/gabarit_officiel.xlsx
@@ -1478,7 +1478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:GG4"/>
+  <dimension ref="A1:GH4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" min="6" max="187"/>
@@ -1589,17 +1589,17 @@
       <c r="CS1" s="1" t="n"/>
       <c r="CT1" s="1" t="n"/>
       <c r="CU1" s="1" t="n"/>
-      <c r="CV1" s="4" t="n"/>
-      <c r="CW1" s="1" t="n"/>
+      <c r="CV1" s="1" t="n"/>
+      <c r="CW1" s="4" t="n"/>
       <c r="CX1" s="1" t="n"/>
       <c r="CY1" s="1" t="n"/>
       <c r="CZ1" s="1" t="n"/>
       <c r="DA1" s="1" t="n"/>
       <c r="DB1" s="1" t="n"/>
-      <c r="DC1" s="5" t="n"/>
-      <c r="DD1" s="1" t="n"/>
+      <c r="DC1" s="1" t="n"/>
+      <c r="DD1" s="5" t="n"/>
       <c r="DE1" s="1" t="n"/>
-      <c r="DF1" s="5" t="n"/>
+      <c r="DF1" s="1" t="n"/>
       <c r="DG1" s="5" t="n"/>
       <c r="DH1" s="5" t="n"/>
       <c r="DI1" s="5" t="n"/>
@@ -1616,27 +1616,27 @@
       <c r="DT1" s="5" t="n"/>
       <c r="DU1" s="5" t="n"/>
       <c r="DV1" s="5" t="n"/>
-      <c r="DW1" s="82" t="n"/>
-      <c r="DX1" s="5" t="n"/>
+      <c r="DW1" s="5" t="n"/>
+      <c r="DX1" s="82" t="n"/>
       <c r="DY1" s="5" t="n"/>
       <c r="DZ1" s="5" t="n"/>
       <c r="EA1" s="5" t="n"/>
-      <c r="EB1" s="1" t="n"/>
-      <c r="EC1" s="5" t="n"/>
-      <c r="ED1" s="1" t="n"/>
+      <c r="EB1" s="5" t="n"/>
+      <c r="EC1" s="1" t="n"/>
+      <c r="ED1" s="5" t="n"/>
       <c r="EE1" s="1" t="n"/>
       <c r="EF1" s="1" t="n"/>
       <c r="EG1" s="1" t="n"/>
       <c r="EH1" s="1" t="n"/>
-      <c r="EI1" s="5" t="n"/>
+      <c r="EI1" s="1" t="n"/>
       <c r="EJ1" s="5" t="n"/>
       <c r="EK1" s="5" t="n"/>
-      <c r="EL1" s="5" t="inlineStr">
+      <c r="EL1" s="5" t="n"/>
+      <c r="EM1" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                              </t>
         </is>
       </c>
-      <c r="EM1" s="5" t="n"/>
       <c r="EN1" s="5" t="n"/>
       <c r="EO1" s="5" t="n"/>
       <c r="EP1" s="5" t="n"/>
@@ -1654,29 +1654,30 @@
       <c r="FB1" s="5" t="n"/>
       <c r="FC1" s="5" t="n"/>
       <c r="FD1" s="5" t="n"/>
-      <c r="FE1" s="6" t="n"/>
-      <c r="FF1" s="5" t="n"/>
+      <c r="FE1" s="5" t="n"/>
+      <c r="FF1" s="6" t="n"/>
       <c r="FG1" s="5" t="n"/>
       <c r="FH1" s="5" t="n"/>
       <c r="FI1" s="5" t="n"/>
       <c r="FJ1" s="5" t="n"/>
       <c r="FK1" s="5" t="n"/>
-      <c r="FL1" s="1" t="n"/>
+      <c r="FL1" s="5" t="n"/>
       <c r="FM1" s="1" t="n"/>
       <c r="FN1" s="1" t="n"/>
       <c r="FO1" s="1" t="n"/>
-      <c r="FP1" s="5" t="n"/>
-      <c r="FQ1" s="1" t="n"/>
+      <c r="FP1" s="1" t="n"/>
+      <c r="FQ1" s="5" t="n"/>
       <c r="FR1" s="1" t="n"/>
       <c r="FS1" s="1" t="n"/>
       <c r="FT1" s="1" t="n"/>
-      <c r="FU1" s="5" t="n"/>
-      <c r="FV1" s="1" t="n"/>
+      <c r="FU1" s="1" t="n"/>
+      <c r="FV1" s="5" t="n"/>
       <c r="FW1" s="1" t="n"/>
       <c r="FX1" s="1" t="n"/>
       <c r="FY1" s="1" t="n"/>
-      <c r="GF1" s="5" t="n"/>
-      <c r="GG1" s="1" t="n"/>
+      <c r="FZ1" s="1" t="n"/>
+      <c r="GG1" s="5" t="n"/>
+      <c r="GH1" s="1" t="n"/>
     </row>
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
@@ -1734,28 +1735,28 @@
       <c r="AC2" s="10" t="n"/>
       <c r="AD2" s="10" t="n"/>
       <c r="AE2" s="10" t="n"/>
-      <c r="AF2" s="9" t="inlineStr">
+      <c r="AF2" s="10" t="n"/>
+      <c r="AG2" s="9" t="inlineStr">
         <is>
           <t>Plans d'exécution spatiaux (Région) (Ruimtelijke uitvoeringsplannen RUP- Gewest)</t>
         </is>
       </c>
-      <c r="AG2" s="11" t="inlineStr">
+      <c r="AH2" s="11" t="inlineStr">
         <is>
           <t>Chercher commune par commune https://dsi.omgeving.vlaanderen.be/fiche-overzicht?locatie=41002 + indiquer le lien vers le RUP</t>
         </is>
       </c>
-      <c r="AH2" s="1" t="n"/>
       <c r="AI2" s="1" t="n"/>
-      <c r="AJ2" s="12" t="n"/>
+      <c r="AJ2" s="1" t="n"/>
       <c r="AK2" s="12" t="n"/>
       <c r="AL2" s="12" t="n"/>
       <c r="AM2" s="12" t="n"/>
-      <c r="AN2" s="13" t="n"/>
+      <c r="AN2" s="12" t="n"/>
       <c r="AO2" s="13" t="n"/>
       <c r="AP2" s="13" t="n"/>
       <c r="AQ2" s="13" t="n"/>
-      <c r="AR2" s="14" t="n"/>
-      <c r="AS2" s="1" t="n"/>
+      <c r="AR2" s="13" t="n"/>
+      <c r="AS2" s="14" t="n"/>
       <c r="AT2" s="1" t="n"/>
       <c r="AU2" s="1" t="n"/>
       <c r="AV2" s="1" t="n"/>
@@ -1767,19 +1768,19 @@
       <c r="BB2" s="1" t="n"/>
       <c r="BC2" s="1" t="n"/>
       <c r="BD2" s="1" t="n"/>
-      <c r="BE2" s="9" t="inlineStr">
+      <c r="BE2" s="1" t="n"/>
+      <c r="BF2" s="9" t="inlineStr">
         <is>
           <t>Plans d'exécution spatiaux (Province) (Ruimtelijke uitvoeringsplannen RUP- Provincie)</t>
         </is>
       </c>
-      <c r="BF2" s="11" t="inlineStr">
+      <c r="BG2" s="11" t="inlineStr">
         <is>
           <t>Chercher commune par commune https://dsi.omgeving.vlaanderen.be/fiche-overzicht?locatie=41002 + indiquer le lien vers le RUP</t>
         </is>
       </c>
-      <c r="BG2" s="1" t="n"/>
       <c r="BH2" s="1" t="n"/>
-      <c r="BI2" s="4" t="n"/>
+      <c r="BI2" s="1" t="n"/>
       <c r="BJ2" s="4" t="n"/>
       <c r="BK2" s="4" t="n"/>
       <c r="BL2" s="4" t="n"/>
@@ -1799,20 +1800,20 @@
       <c r="BZ2" s="4" t="n"/>
       <c r="CA2" s="4" t="n"/>
       <c r="CB2" s="4" t="n"/>
-      <c r="CC2" s="15" t="n"/>
-      <c r="CD2" s="9" t="inlineStr">
+      <c r="CC2" s="4" t="n"/>
+      <c r="CD2" s="15" t="n"/>
+      <c r="CE2" s="9" t="inlineStr">
         <is>
           <t>Plans d'exécution spatiaux (Commune) (Ruimtelijke uitvoeringsplannen RUP- Gemeente)</t>
         </is>
       </c>
-      <c r="CE2" s="11" t="inlineStr">
+      <c r="CF2" s="11" t="inlineStr">
         <is>
           <t>Chercher commune par commune https://dsi.omgeving.vlaanderen.be/fiche-overzicht?locatie=41002 + indiquer le lien vers le RUP</t>
         </is>
       </c>
-      <c r="CF2" s="1" t="n"/>
       <c r="CG2" s="1" t="n"/>
-      <c r="CH2" s="15" t="n"/>
+      <c r="CH2" s="1" t="n"/>
       <c r="CI2" s="15" t="n"/>
       <c r="CJ2" s="15" t="n"/>
       <c r="CK2" s="15" t="n"/>
@@ -1830,26 +1831,26 @@
       <c r="CW2" s="15" t="n"/>
       <c r="CX2" s="15" t="n"/>
       <c r="CY2" s="15" t="n"/>
-      <c r="CZ2" s="16" t="n"/>
-      <c r="DA2" s="9" t="n"/>
+      <c r="CZ2" s="15" t="n"/>
+      <c r="DA2" s="16" t="n"/>
       <c r="DB2" s="9" t="n"/>
-      <c r="DC2" s="9" t="inlineStr">
+      <c r="DC2" s="9" t="n"/>
+      <c r="DD2" s="9" t="inlineStr">
         <is>
           <t>Inondation (Watertoets)</t>
         </is>
       </c>
-      <c r="DD2" s="1" t="n"/>
-      <c r="DE2" s="17" t="inlineStr">
+      <c r="DE2" s="1" t="n"/>
+      <c r="DF2" s="17" t="inlineStr">
         <is>
           <t>natur et milieu ( milieu)</t>
         </is>
       </c>
-      <c r="DF2" s="134" t="inlineStr">
+      <c r="DG2" s="134" t="inlineStr">
         <is>
           <t>natur et milieu ( milieu)</t>
         </is>
       </c>
-      <c r="DG2" s="135" t="n"/>
       <c r="DH2" s="135" t="n"/>
       <c r="DI2" s="135" t="n"/>
       <c r="DJ2" s="135" t="n"/>
@@ -1859,238 +1860,239 @@
       <c r="DN2" s="135" t="n"/>
       <c r="DO2" s="135" t="n"/>
       <c r="DP2" s="135" t="n"/>
-      <c r="DQ2" s="136" t="n"/>
-      <c r="DR2" s="120" t="n"/>
+      <c r="DQ2" s="135" t="n"/>
+      <c r="DR2" s="136" t="n"/>
       <c r="DS2" s="120" t="n"/>
       <c r="DT2" s="120" t="n"/>
       <c r="DU2" s="120" t="n"/>
-      <c r="DV2" s="17" t="inlineStr">
+      <c r="DV2" s="120" t="n"/>
+      <c r="DW2" s="17" t="inlineStr">
         <is>
           <t>natur et milieu (WATER)</t>
         </is>
       </c>
-      <c r="DW2" s="17" t="inlineStr">
+      <c r="DX2" s="17" t="inlineStr">
         <is>
           <t>natur et milieu (WATER)</t>
         </is>
       </c>
-      <c r="DX2" s="17" t="inlineStr">
+      <c r="DY2" s="17" t="inlineStr">
         <is>
           <t>natur et milieu (WATER)</t>
         </is>
       </c>
-      <c r="DY2" s="17" t="inlineStr">
+      <c r="DZ2" s="17" t="inlineStr">
         <is>
           <t>natur et milieu (WATER)</t>
         </is>
       </c>
-      <c r="DZ2" s="17" t="inlineStr">
+      <c r="EA2" s="17" t="inlineStr">
         <is>
           <t>natur et milieu (WATER)</t>
         </is>
       </c>
-      <c r="EA2" s="17" t="inlineStr">
+      <c r="EB2" s="17" t="inlineStr">
         <is>
           <t>natur et milieu (WATER)</t>
         </is>
       </c>
-      <c r="EB2" s="17" t="inlineStr">
+      <c r="EC2" s="17" t="inlineStr">
         <is>
           <t>natur et milieu (WATER)</t>
         </is>
       </c>
-      <c r="EC2" s="18" t="inlineStr">
+      <c r="ED2" s="18" t="inlineStr">
         <is>
           <t>Natuur en milieu (BODEM)</t>
         </is>
       </c>
-      <c r="ED2" s="1" t="n"/>
       <c r="EE2" s="1" t="n"/>
       <c r="EF2" s="1" t="n"/>
       <c r="EG2" s="1" t="n"/>
       <c r="EH2" s="1" t="n"/>
-      <c r="EI2" s="17" t="inlineStr">
+      <c r="EI2" s="1" t="n"/>
+      <c r="EJ2" s="17" t="inlineStr">
         <is>
           <t>BODEM
  (Erosiegevoeligheidskaart)</t>
         </is>
       </c>
-      <c r="EJ2" s="18" t="inlineStr">
+      <c r="EK2" s="18" t="inlineStr">
         <is>
           <t>BODEM</t>
         </is>
       </c>
-      <c r="EK2" s="18" t="inlineStr">
+      <c r="EL2" s="18" t="inlineStr">
         <is>
           <t>BODEM</t>
         </is>
       </c>
-      <c r="EL2" s="18" t="inlineStr">
+      <c r="EM2" s="18" t="inlineStr">
         <is>
           <t>BODEM</t>
         </is>
       </c>
-      <c r="EM2" s="17" t="inlineStr">
+      <c r="EN2" s="17" t="inlineStr">
         <is>
           <t>BODEM
 (Watertoets: advieskaart, 2023)</t>
         </is>
       </c>
-      <c r="EN2" s="19" t="inlineStr">
+      <c r="EO2" s="19" t="inlineStr">
         <is>
           <t>Economie ( bedrijven)</t>
         </is>
       </c>
-      <c r="EO2" s="18" t="inlineStr">
+      <c r="EP2" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve"> ( bedrijven)</t>
         </is>
       </c>
-      <c r="EP2" s="18" t="inlineStr">
+      <c r="EQ2" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve"> ( bedrijven)</t>
         </is>
       </c>
-      <c r="EQ2" s="18" t="inlineStr">
+      <c r="ER2" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve"> ( bedrijven)</t>
         </is>
       </c>
-      <c r="ER2" s="18" t="inlineStr">
+      <c r="ES2" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve"> ( bedrijven)</t>
         </is>
       </c>
-      <c r="ES2" s="18" t="inlineStr">
+      <c r="ET2" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve"> ( bedrijven)</t>
         </is>
       </c>
-      <c r="ET2" s="17" t="inlineStr">
+      <c r="EU2" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve"> ( bedrijven)
 (Steunzones - Gebieden waar inhouding van bedrijfsvoorheffing mogelijk is)</t>
         </is>
       </c>
-      <c r="EU2" s="18" t="inlineStr">
+      <c r="EV2" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve"> ( bedrijven)</t>
         </is>
       </c>
-      <c r="EV2" s="18" t="inlineStr">
+      <c r="EW2" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve"> ( bedrijven)</t>
         </is>
       </c>
-      <c r="EW2" s="9" t="inlineStr">
+      <c r="EX2" s="9" t="inlineStr">
         <is>
           <t>Natuur en milieu</t>
         </is>
       </c>
-      <c r="EX2" s="18" t="inlineStr">
+      <c r="EY2" s="18" t="inlineStr">
         <is>
           <t>Landinrichting</t>
         </is>
       </c>
-      <c r="EY2" s="18" t="inlineStr">
+      <c r="EZ2" s="18" t="inlineStr">
         <is>
           <t>Landinrichting</t>
         </is>
       </c>
-      <c r="EZ2" s="18" t="inlineStr">
+      <c r="FA2" s="18" t="inlineStr">
         <is>
           <t>Landinrichting</t>
         </is>
       </c>
-      <c r="FA2" s="20" t="inlineStr">
+      <c r="FB2" s="20" t="inlineStr">
         <is>
           <t>Landinrichting
 Ruilverkaveling van landeigendommen uit kracht van wet</t>
         </is>
       </c>
-      <c r="FB2" s="9" t="inlineStr">
+      <c r="FC2" s="9" t="inlineStr">
         <is>
           <t>Natuur en milieu (Landschap)</t>
         </is>
       </c>
-      <c r="FC2" s="9" t="n"/>
-      <c r="FD2" s="17" t="inlineStr">
+      <c r="FD2" s="9" t="n"/>
+      <c r="FE2" s="17" t="inlineStr">
         <is>
           <t>Natuur en milieu ( Milieu)
 Natura 2000 Habitatkaart</t>
         </is>
       </c>
-      <c r="FE2" s="17" t="inlineStr">
+      <c r="FF2" s="17" t="inlineStr">
         <is>
           <t>Natuur en milieu ( Natur) Natuurbeheerplannen
 Bosreferentielaag 2000</t>
         </is>
       </c>
-      <c r="FF2" s="1" t="n"/>
-      <c r="FG2" s="17" t="inlineStr">
+      <c r="FG2" s="1" t="n"/>
+      <c r="FH2" s="17" t="inlineStr">
         <is>
           <t>Natur en milieu ( Natur)</t>
         </is>
       </c>
-      <c r="FH2" s="17" t="inlineStr">
+      <c r="FI2" s="17" t="inlineStr">
         <is>
           <t>Natur en milieu ( Natur)
 VEN en het IVON</t>
         </is>
       </c>
-      <c r="FI2" s="17" t="inlineStr">
+      <c r="FJ2" s="17" t="inlineStr">
         <is>
           <t>Natur en milieu ( Natur)</t>
         </is>
       </c>
-      <c r="FJ2" s="17" t="inlineStr">
+      <c r="FK2" s="17" t="inlineStr">
         <is>
           <t>Natur en milieu ( Natur)</t>
         </is>
       </c>
-      <c r="FK2" s="17" t="inlineStr">
+      <c r="FL2" s="17" t="inlineStr">
         <is>
           <t>Bouwen en wonen ( Geluidsbelasting)</t>
         </is>
       </c>
-      <c r="FL2" s="21" t="n"/>
       <c r="FM2" s="21" t="n"/>
       <c r="FN2" s="21" t="n"/>
       <c r="FO2" s="21" t="n"/>
-      <c r="FP2" s="17" t="inlineStr">
+      <c r="FP2" s="21" t="n"/>
+      <c r="FQ2" s="17" t="inlineStr">
         <is>
           <t>Bouwen en wonen ( Geluidsbelasting)</t>
         </is>
       </c>
-      <c r="FQ2" s="21" t="n"/>
       <c r="FR2" s="21" t="n"/>
       <c r="FS2" s="21" t="n"/>
       <c r="FT2" s="21" t="n"/>
-      <c r="FU2" s="17" t="inlineStr">
+      <c r="FU2" s="21" t="n"/>
+      <c r="FV2" s="17" t="inlineStr">
         <is>
           <t>Bouwen en wonen ( Geluidsbelasting)</t>
         </is>
       </c>
-      <c r="FV2" s="22" t="n"/>
       <c r="FW2" s="22" t="n"/>
       <c r="FX2" s="22" t="n"/>
       <c r="FY2" s="22" t="n"/>
-      <c r="FZ2" s="9" t="inlineStr">
+      <c r="FZ2" s="22" t="n"/>
+      <c r="GA2" s="9" t="inlineStr">
         <is>
           <t>Etat des sols -mj https://www.degrotegrondvraag.be/</t>
         </is>
       </c>
-      <c r="GA2" s="22" t="n"/>
       <c r="GB2" s="22" t="n"/>
       <c r="GC2" s="22" t="n"/>
       <c r="GD2" s="22" t="n"/>
       <c r="GE2" s="22" t="n"/>
-      <c r="GF2" s="9" t="inlineStr">
+      <c r="GF2" s="22" t="n"/>
+      <c r="GG2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve"> Code du logement (Bouwen en wonen ,Vlaamse wooncode)</t>
         </is>
       </c>
-      <c r="GG2" s="9" t="n"/>
+      <c r="GH2" s="9" t="n"/>
     </row>
     <row r="3" ht="63.75" customHeight="1">
       <c r="A3" s="23" t="n"/>
@@ -2228,692 +2230,697 @@
           <t>Gebieden voor dagrecreatie</t>
         </is>
       </c>
-      <c r="AF3" s="41" t="inlineStr">
+      <c r="AF3" s="102" t="inlineStr">
+        <is>
+          <t>lokaal bedrijventerrein met openbaar karakter</t>
+        </is>
+      </c>
+      <c r="AG3" s="41" t="inlineStr">
         <is>
           <t>Lien plan d'execution REGION</t>
         </is>
       </c>
-      <c r="AG3" s="41" t="inlineStr">
+      <c r="AH3" s="41" t="inlineStr">
         <is>
           <t>RUP</t>
         </is>
       </c>
-      <c r="AH3" s="26" t="inlineStr">
+      <c r="AI3" s="26" t="inlineStr">
         <is>
           <t>Wonen (zone d'habitat)</t>
         </is>
       </c>
-      <c r="AI3" s="26" t="inlineStr">
+      <c r="AJ3" s="26" t="inlineStr">
         <is>
           <t>Zone voor kleinschalig wonen</t>
         </is>
       </c>
-      <c r="AJ3" s="42" t="inlineStr">
+      <c r="AK3" s="42" t="inlineStr">
         <is>
           <t>Bedrijvigheid</t>
         </is>
       </c>
-      <c r="AK3" s="43" t="inlineStr">
+      <c r="AL3" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">Bedrijvigheid - Buffer
 </t>
         </is>
       </c>
-      <c r="AL3" s="38" t="inlineStr">
+      <c r="AM3" s="38" t="inlineStr">
         <is>
           <t>Recreatie</t>
         </is>
       </c>
-      <c r="AM3" s="38" t="inlineStr">
+      <c r="AN3" s="38" t="inlineStr">
         <is>
           <t>Recreatie (Natuurverwerving)</t>
         </is>
       </c>
-      <c r="AN3" s="34" t="inlineStr">
+      <c r="AO3" s="34" t="inlineStr">
         <is>
           <t>Landbouw- agrarisch gebied</t>
         </is>
       </c>
-      <c r="AO3" s="44" t="inlineStr">
+      <c r="AP3" s="44" t="inlineStr">
         <is>
           <t>Landbouw- agrarische bedrijvenzone</t>
         </is>
       </c>
-      <c r="AP3" s="45" t="inlineStr">
+      <c r="AQ3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- bouwvrij agrarisch gebied</t>
         </is>
       </c>
-      <c r="AQ3" s="45" t="inlineStr">
+      <c r="AR3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- Agrarisch gebied met ecologisch belang</t>
         </is>
       </c>
-      <c r="AR3" s="46" t="inlineStr">
+      <c r="AS3" s="46" t="inlineStr">
         <is>
           <t>Bois (Bos)</t>
         </is>
       </c>
-      <c r="AS3" s="47" t="inlineStr">
+      <c r="AT3" s="47" t="inlineStr">
         <is>
           <t>Zone verte (Overig groen - gemengd openruimtegebied)</t>
         </is>
       </c>
-      <c r="AT3" s="47" t="inlineStr">
+      <c r="AU3" s="47" t="inlineStr">
         <is>
           <t>Zone verte (Overig groen- parkgebied)</t>
         </is>
       </c>
-      <c r="AU3" s="47" t="inlineStr">
+      <c r="AV3" s="47" t="inlineStr">
         <is>
           <t>Zone verte - Overig groen-Gemengd openruimtegebied met cultuurhistorische waarde</t>
         </is>
       </c>
-      <c r="AV3" s="47" t="inlineStr">
+      <c r="AW3" s="47" t="inlineStr">
         <is>
           <t>Zone verte- Overig groen -bestaande, vergunde of vergund geachte weekendverblijven</t>
         </is>
       </c>
-      <c r="AW3" s="48" t="inlineStr">
+      <c r="AX3" s="48" t="inlineStr">
         <is>
           <t>Natuurgebied</t>
         </is>
       </c>
-      <c r="AX3" s="48" t="inlineStr">
+      <c r="AY3" s="48" t="inlineStr">
         <is>
           <t>Natuurreservaat</t>
         </is>
       </c>
-      <c r="AY3" s="49" t="inlineStr">
+      <c r="AZ3" s="49" t="inlineStr">
         <is>
           <t>Gemeenschaps- en nutsvoorzieningen</t>
         </is>
       </c>
-      <c r="AZ3" s="49" t="inlineStr">
+      <c r="BA3" s="49" t="inlineStr">
         <is>
           <t>Gebied voor zuiveringsinfrastructuur voor afvalwater</t>
         </is>
       </c>
-      <c r="BA3" s="49" t="inlineStr">
+      <c r="BB3" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">gebied voor infrastructuur voor duurzame watervoorziening </t>
         </is>
       </c>
-      <c r="BB3" s="49" t="inlineStr">
+      <c r="BC3" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">
 gebied voor de winning van oppervlaktedelfstoffen </t>
         </is>
       </c>
-      <c r="BC3" s="49" t="inlineStr">
+      <c r="BD3" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">gebied voor verwerking van oppervlaktedelfstoffen </t>
         </is>
       </c>
-      <c r="BD3" s="50" t="inlineStr">
+      <c r="BE3" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">Gebied voor projectgrindwinning
 </t>
         </is>
       </c>
-      <c r="BE3" s="41" t="inlineStr">
+      <c r="BF3" s="41" t="inlineStr">
         <is>
           <t>Lien plman d'execution PROVINCE</t>
         </is>
       </c>
-      <c r="BF3" s="41" t="inlineStr">
+      <c r="BG3" s="41" t="inlineStr">
         <is>
           <t>RUP</t>
         </is>
       </c>
-      <c r="BG3" s="26" t="inlineStr">
+      <c r="BH3" s="26" t="inlineStr">
         <is>
           <t>Wonen (zone d'habitat)</t>
         </is>
       </c>
-      <c r="BH3" s="26" t="inlineStr">
+      <c r="BI3" s="26" t="inlineStr">
         <is>
           <t>Zone voor kleinschalig wonen</t>
         </is>
       </c>
-      <c r="BI3" s="42" t="inlineStr">
+      <c r="BJ3" s="42" t="inlineStr">
         <is>
           <t>Bedrijvigheid</t>
         </is>
       </c>
-      <c r="BJ3" s="42" t="inlineStr">
+      <c r="BK3" s="42" t="inlineStr">
         <is>
           <t xml:space="preserve">Bedrijvigheid - Buffer
 </t>
         </is>
       </c>
-      <c r="BK3" s="38" t="inlineStr">
+      <c r="BL3" s="38" t="inlineStr">
         <is>
           <t>Recreatie</t>
         </is>
       </c>
-      <c r="BL3" s="38" t="inlineStr">
+      <c r="BM3" s="38" t="inlineStr">
         <is>
           <t>Recreatie (Natuurverwerving)</t>
         </is>
       </c>
-      <c r="BM3" s="34" t="inlineStr">
+      <c r="BN3" s="34" t="inlineStr">
         <is>
           <t>Landbouw- agrarisch gebied</t>
         </is>
       </c>
-      <c r="BN3" s="45" t="inlineStr">
+      <c r="BO3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- agrarische bedrijvenzone</t>
         </is>
       </c>
-      <c r="BO3" s="45" t="inlineStr">
+      <c r="BP3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- bouwvrij agrarisch gebied</t>
         </is>
       </c>
-      <c r="BP3" s="45" t="inlineStr">
+      <c r="BQ3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- Agrarisch gebied met ecologisch belang</t>
         </is>
       </c>
-      <c r="BQ3" s="46" t="inlineStr">
+      <c r="BR3" s="46" t="inlineStr">
         <is>
           <t>Bois (Bos)</t>
         </is>
       </c>
-      <c r="BR3" s="47" t="inlineStr">
+      <c r="BS3" s="47" t="inlineStr">
         <is>
           <t>Zone verte (Overig groen - gemengd openruimtegebied)</t>
         </is>
       </c>
-      <c r="BS3" s="47" t="inlineStr">
+      <c r="BT3" s="47" t="inlineStr">
         <is>
           <t>Zone verte (Overig groen- parkgebied)</t>
         </is>
       </c>
-      <c r="BT3" s="47" t="inlineStr">
+      <c r="BU3" s="47" t="inlineStr">
         <is>
           <t>Zone verte - Overig groen-Gemengd openruimtegebied met cultuurhistorische waarde</t>
         </is>
       </c>
-      <c r="BU3" s="47" t="inlineStr">
+      <c r="BV3" s="47" t="inlineStr">
         <is>
           <t>Zone verte- Overig groen -bestaande, vergunde of vergund geachte weekendverblijven</t>
         </is>
       </c>
-      <c r="BV3" s="48" t="inlineStr">
+      <c r="BW3" s="48" t="inlineStr">
         <is>
           <t>Natuurgebied</t>
         </is>
       </c>
-      <c r="BW3" s="48" t="inlineStr">
+      <c r="BX3" s="48" t="inlineStr">
         <is>
           <t>Natuurreservaat</t>
         </is>
       </c>
-      <c r="BX3" s="49" t="inlineStr">
+      <c r="BY3" s="49" t="inlineStr">
         <is>
           <t>Gemeenschaps- en nutsvoorzieningen</t>
         </is>
       </c>
-      <c r="BY3" s="49" t="inlineStr">
+      <c r="BZ3" s="49" t="inlineStr">
         <is>
           <t>Gebied voor zuiveringsinfrastructuur voor afvalwater</t>
         </is>
       </c>
-      <c r="BZ3" s="49" t="inlineStr">
+      <c r="CA3" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">gebied voor infrastructuur voor duurzame watervoorziening </t>
         </is>
       </c>
-      <c r="CA3" s="49" t="inlineStr">
+      <c r="CB3" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">
 gebied voor de winning van oppervlaktedelfstoffen </t>
         </is>
       </c>
-      <c r="CB3" s="49" t="inlineStr">
+      <c r="CC3" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">gebied voor verwerking van oppervlaktedelfstoffen </t>
         </is>
       </c>
-      <c r="CC3" s="50" t="inlineStr">
+      <c r="CD3" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">Gebied voor projectgrindwinning
 </t>
         </is>
       </c>
-      <c r="CD3" s="41" t="inlineStr">
+      <c r="CE3" s="41" t="inlineStr">
         <is>
           <t>Lien  d'execution commune</t>
         </is>
       </c>
-      <c r="CE3" s="41" t="inlineStr">
+      <c r="CF3" s="41" t="inlineStr">
         <is>
           <t>RUP</t>
         </is>
       </c>
-      <c r="CF3" s="26" t="inlineStr">
+      <c r="CG3" s="26" t="inlineStr">
         <is>
           <t>Wonen (zone d'habitat)</t>
         </is>
       </c>
-      <c r="CG3" s="26" t="inlineStr">
+      <c r="CH3" s="26" t="inlineStr">
         <is>
           <t>Zone voor kleinschalig wonen</t>
         </is>
       </c>
-      <c r="CH3" s="42" t="inlineStr">
+      <c r="CI3" s="42" t="inlineStr">
         <is>
           <t>Bedrijvigheid</t>
         </is>
       </c>
-      <c r="CI3" s="51" t="inlineStr">
+      <c r="CJ3" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Bedrijvigheid - Buffer
 </t>
         </is>
       </c>
-      <c r="CJ3" s="38" t="inlineStr">
+      <c r="CK3" s="38" t="inlineStr">
         <is>
           <t>Recreatie</t>
         </is>
       </c>
-      <c r="CK3" s="38" t="inlineStr">
+      <c r="CL3" s="38" t="inlineStr">
         <is>
           <t>Recreatie (Natuurverwerving)</t>
         </is>
       </c>
-      <c r="CL3" s="45" t="inlineStr">
+      <c r="CM3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- agrarisch gebied</t>
         </is>
       </c>
-      <c r="CM3" s="45" t="inlineStr">
+      <c r="CN3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- agrarische bedrijvenzone</t>
         </is>
       </c>
-      <c r="CN3" s="45" t="inlineStr">
+      <c r="CO3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- bouwvrij agrarisch gebied</t>
         </is>
       </c>
-      <c r="CO3" s="45" t="inlineStr">
+      <c r="CP3" s="45" t="inlineStr">
         <is>
           <t>Landbouw- Agrarisch gebied met ecologisch belang</t>
         </is>
       </c>
-      <c r="CP3" s="46" t="inlineStr">
+      <c r="CQ3" s="46" t="inlineStr">
         <is>
           <t>Bois (Bos)</t>
         </is>
       </c>
-      <c r="CQ3" s="47" t="inlineStr">
+      <c r="CR3" s="47" t="inlineStr">
         <is>
           <t>Zone verte (Overig groen - gemengd openruimtegebied)</t>
         </is>
       </c>
-      <c r="CR3" s="47" t="inlineStr">
+      <c r="CS3" s="47" t="inlineStr">
         <is>
           <t>Zone verte (Overig groen- parkgebied)</t>
         </is>
       </c>
-      <c r="CS3" s="47" t="inlineStr">
+      <c r="CT3" s="47" t="inlineStr">
         <is>
           <t>Zone verte - Overig groen-Gemengd openruimtegebied met cultuurhistorische waarde</t>
         </is>
       </c>
-      <c r="CT3" s="47" t="inlineStr">
+      <c r="CU3" s="47" t="inlineStr">
         <is>
           <t>Zone verte- Overig groen -bestaande, vergunde of vergund geachte weekendverblijven</t>
         </is>
       </c>
-      <c r="CU3" s="48" t="inlineStr">
+      <c r="CV3" s="48" t="inlineStr">
         <is>
           <t>Natuurgebied</t>
         </is>
       </c>
-      <c r="CV3" s="48" t="inlineStr">
+      <c r="CW3" s="48" t="inlineStr">
         <is>
           <t>Natuurreservaat</t>
         </is>
       </c>
-      <c r="CW3" s="49" t="inlineStr">
+      <c r="CX3" s="49" t="inlineStr">
         <is>
           <t>Gemeenschaps- en nutsvoorzieningen</t>
         </is>
       </c>
-      <c r="CX3" s="49" t="inlineStr">
+      <c r="CY3" s="49" t="inlineStr">
         <is>
           <t>Gebied voor zuiveringsinfrastructuur voor afvalwater</t>
         </is>
       </c>
-      <c r="CY3" s="49" t="inlineStr">
+      <c r="CZ3" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">gebied voor infrastructuur voor duurzame watervoorziening </t>
         </is>
       </c>
-      <c r="CZ3" s="52" t="inlineStr">
+      <c r="DA3" s="52" t="inlineStr">
         <is>
           <t xml:space="preserve">
 gebied voor de winning van oppervlaktedelfstoffen </t>
         </is>
       </c>
-      <c r="DA3" s="49" t="inlineStr">
+      <c r="DB3" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">gebied voor verwerking van oppervlaktedelfstoffen </t>
         </is>
       </c>
-      <c r="DB3" s="50" t="inlineStr">
+      <c r="DC3" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">Gebied voor projectgrindwinning
 </t>
         </is>
       </c>
-      <c r="DC3" s="103" t="inlineStr">
+      <c r="DD3" s="103" t="inlineStr">
         <is>
           <t>Mogelijk overstromingsgevoelig</t>
         </is>
       </c>
-      <c r="DD3" s="53" t="inlineStr">
+      <c r="DE3" s="53" t="inlineStr">
         <is>
           <t>Effectief overstromingsgevoelig</t>
         </is>
       </c>
-      <c r="DE3" s="54" t="inlineStr">
+      <c r="DF3" s="54" t="inlineStr">
         <is>
           <t>Beheergebieden beheerovereenkomst waterwaliteit</t>
         </is>
       </c>
-      <c r="DF3" s="121" t="inlineStr">
+      <c r="DG3" s="121" t="inlineStr">
         <is>
           <t>Overstromingsgevoelige gebieden  Pluvial</t>
         </is>
       </c>
-      <c r="DG3" s="137" t="n"/>
       <c r="DH3" s="137" t="n"/>
       <c r="DI3" s="137" t="n"/>
-      <c r="DJ3" s="121" t="inlineStr">
+      <c r="DJ3" s="137" t="n"/>
+      <c r="DK3" s="121" t="inlineStr">
         <is>
           <t xml:space="preserve">Overstromingsgevoelige gebieden Fluvial </t>
         </is>
       </c>
-      <c r="DK3" s="137" t="n"/>
       <c r="DL3" s="137" t="n"/>
       <c r="DM3" s="137" t="n"/>
-      <c r="DN3" s="123" t="inlineStr">
+      <c r="DN3" s="137" t="n"/>
+      <c r="DO3" s="123" t="inlineStr">
         <is>
           <t>Overstromingsgevoelige gebieden vanuit zee</t>
         </is>
       </c>
-      <c r="DO3" s="137" t="n"/>
       <c r="DP3" s="137" t="n"/>
-      <c r="DQ3" s="138" t="n"/>
-      <c r="DR3" s="139" t="inlineStr">
+      <c r="DQ3" s="137" t="n"/>
+      <c r="DR3" s="138" t="n"/>
+      <c r="DS3" s="139" t="inlineStr">
         <is>
           <t>Afgebakende overstromingsgebieden en oeverzones</t>
         </is>
       </c>
-      <c r="DS3" s="138" t="n"/>
-      <c r="DT3" s="139" t="inlineStr">
+      <c r="DT3" s="138" t="n"/>
+      <c r="DU3" s="139" t="inlineStr">
         <is>
           <t>Signaalgebieden</t>
         </is>
       </c>
-      <c r="DU3" s="138" t="n"/>
-      <c r="DV3" s="55" t="inlineStr">
+      <c r="DV3" s="138" t="n"/>
+      <c r="DW3" s="55" t="inlineStr">
         <is>
           <t>Grond waterstromingsgevoelige gebieden</t>
         </is>
       </c>
-      <c r="DW3" s="56" t="inlineStr">
+      <c r="DX3" s="56" t="inlineStr">
         <is>
           <t>Van Natuur overstroombare gebieden</t>
         </is>
       </c>
-      <c r="DX3" s="57" t="inlineStr">
+      <c r="DY3" s="57" t="inlineStr">
         <is>
           <t>Risicozones voor overstromingen: nieuwe en bevestigde risocozones</t>
         </is>
       </c>
-      <c r="DY3" s="58" t="inlineStr">
+      <c r="DZ3" s="58" t="inlineStr">
         <is>
           <t>Recent overstromde gebieden</t>
         </is>
       </c>
-      <c r="DZ3" s="59" t="inlineStr">
+      <c r="EA3" s="59" t="inlineStr">
         <is>
           <t>Overstromingsgebieden en oeverzones - integraal waterbeleid</t>
         </is>
       </c>
-      <c r="EA3" s="60" t="inlineStr">
+      <c r="EB3" s="60" t="inlineStr">
         <is>
           <t>Grondwaterwingebieden en beschermingszones</t>
         </is>
       </c>
-      <c r="EB3" s="61" t="inlineStr">
+      <c r="EC3" s="61" t="inlineStr">
         <is>
           <t>Infiltratiegevoelige bodems</t>
         </is>
       </c>
-      <c r="EC3" s="59" t="inlineStr">
+      <c r="ED3" s="59" t="inlineStr">
         <is>
           <t>Afstromingskaart (enkelvoudige stroomlijnen)</t>
         </is>
       </c>
-      <c r="ED3" s="59" t="n"/>
       <c r="EE3" s="59" t="n"/>
       <c r="EF3" s="59" t="n"/>
       <c r="EG3" s="59" t="n"/>
       <c r="EH3" s="59" t="n"/>
-      <c r="EI3" s="104" t="inlineStr">
+      <c r="EI3" s="59" t="n"/>
+      <c r="EJ3" s="104" t="inlineStr">
         <is>
           <t>Andere erosiegerelateerde gronden</t>
         </is>
       </c>
-      <c r="EJ3" s="57" t="inlineStr">
+      <c r="EK3" s="57" t="inlineStr">
         <is>
           <t>Gekarteerde grondverschuivingen</t>
         </is>
       </c>
-      <c r="EK3" s="62" t="inlineStr">
+      <c r="EL3" s="62" t="inlineStr">
         <is>
           <t>Gevoeligheid voor grondverschuivingen</t>
         </is>
       </c>
-      <c r="EL3" s="63" t="inlineStr">
+      <c r="EM3" s="63" t="inlineStr">
         <is>
           <t>Potentiële bodemerosiekaart per perceel 2021</t>
         </is>
       </c>
-      <c r="EM3" s="64" t="inlineStr">
+      <c r="EN3" s="64" t="inlineStr">
         <is>
           <t>Watertoets</t>
         </is>
       </c>
-      <c r="EN3" s="65" t="inlineStr">
+      <c r="EO3" s="65" t="inlineStr">
         <is>
           <t>Aangeboden bedrijventerreinperceel</t>
         </is>
       </c>
-      <c r="EO3" s="60" t="inlineStr">
+      <c r="EP3" s="60" t="inlineStr">
         <is>
           <t>Bedrijventerrein</t>
         </is>
       </c>
-      <c r="EP3" s="60" t="inlineStr">
+      <c r="EQ3" s="60" t="inlineStr">
         <is>
           <t>Beheerde bedrijvenzone</t>
         </is>
       </c>
-      <c r="EQ3" s="66" t="inlineStr">
+      <c r="ER3" s="66" t="inlineStr">
         <is>
           <t>Ontwikkelbare bedrijvenzone</t>
         </is>
       </c>
-      <c r="ER3" s="19" t="inlineStr">
+      <c r="ES3" s="19" t="inlineStr">
         <is>
           <t>Planningszone met economische bestemming</t>
         </is>
       </c>
-      <c r="ES3" s="67" t="inlineStr">
+      <c r="ET3" s="67" t="inlineStr">
         <is>
           <t>Brownfieldconvenanten</t>
         </is>
       </c>
-      <c r="ET3" s="60" t="inlineStr">
+      <c r="EU3" s="60" t="inlineStr">
         <is>
           <t>Steunzone</t>
         </is>
       </c>
-      <c r="EU3" s="68" t="inlineStr">
+      <c r="EV3" s="68" t="inlineStr">
         <is>
           <t>Seveso inrichingen</t>
         </is>
       </c>
-      <c r="EV3" s="69" t="inlineStr">
+      <c r="EW3" s="69" t="inlineStr">
         <is>
           <t>Consultatie zone van Seveso-inrichtingen</t>
         </is>
       </c>
-      <c r="EW3" s="44" t="inlineStr">
+      <c r="EX3" s="44" t="inlineStr">
         <is>
           <t>Landinrichting in onderzoek</t>
         </is>
       </c>
-      <c r="EX3" s="70" t="inlineStr">
+      <c r="EY3" s="70" t="inlineStr">
         <is>
           <t>Vastgesteld landinrichtingsproject</t>
         </is>
       </c>
-      <c r="EY3" s="71" t="inlineStr">
+      <c r="EZ3" s="71" t="inlineStr">
         <is>
           <t>Landinrichtingsplan</t>
         </is>
       </c>
-      <c r="EZ3" s="36" t="inlineStr">
+      <c r="FA3" s="36" t="inlineStr">
         <is>
           <t>Natuurinrichting</t>
         </is>
       </c>
-      <c r="FA3" s="26" t="inlineStr">
+      <c r="FB3" s="26" t="inlineStr">
         <is>
           <t>Ruilverkaveling
 (Ruilverkaveling van landeigendommen uit kracht van wet)</t>
         </is>
       </c>
-      <c r="FB3" s="72" t="inlineStr">
+      <c r="FC3" s="72" t="inlineStr">
         <is>
           <t>Fysische systeemeenheden</t>
         </is>
       </c>
-      <c r="FC3" s="73" t="inlineStr">
+      <c r="FD3" s="73" t="inlineStr">
         <is>
           <t>Traditionele landschappen</t>
         </is>
       </c>
-      <c r="FD3" s="62" t="inlineStr">
+      <c r="FE3" s="62" t="inlineStr">
         <is>
           <t>Beheergebieden Natura 2000-soorten</t>
         </is>
       </c>
-      <c r="FE3" s="74" t="inlineStr">
+      <c r="FF3" s="74" t="inlineStr">
         <is>
           <t>Bosreservaten</t>
         </is>
       </c>
-      <c r="FF3" s="66" t="inlineStr">
+      <c r="FG3" s="66" t="inlineStr">
         <is>
           <t>Erkende Natuurreservaten</t>
         </is>
       </c>
-      <c r="FG3" s="62" t="inlineStr">
+      <c r="FH3" s="62" t="inlineStr">
         <is>
           <t>Gebieden duinendecreet</t>
         </is>
       </c>
-      <c r="FH3" s="75" t="inlineStr">
+      <c r="FI3" s="75" t="inlineStr">
         <is>
           <t>Gebieden van het VEN en het IVON
 (VEN en het IVON)</t>
         </is>
       </c>
-      <c r="FI3" s="76" t="inlineStr">
+      <c r="FJ3" s="76" t="inlineStr">
         <is>
           <t>Habitatrichtlijngebieden</t>
         </is>
       </c>
-      <c r="FJ3" s="77" t="inlineStr">
+      <c r="FK3" s="77" t="inlineStr">
         <is>
           <t>Vogelrichtlijngebieden</t>
         </is>
       </c>
-      <c r="FK3" s="21" t="inlineStr">
+      <c r="FL3" s="21" t="inlineStr">
         <is>
           <t>Geluidsbelasting belangrijke wegen Lnight 2021
   (Exposition au bruit- routes)</t>
         </is>
       </c>
-      <c r="FL3" s="1" t="n"/>
       <c r="FM3" s="1" t="n"/>
       <c r="FN3" s="1" t="n"/>
       <c r="FO3" s="1" t="n"/>
-      <c r="FP3" s="21" t="inlineStr">
+      <c r="FP3" s="1" t="n"/>
+      <c r="FQ3" s="21" t="inlineStr">
         <is>
           <t>Geluidsbelasting belangrijke luchthaven(s) Lnight 2021(Exposition au bruit- voies ferrées)</t>
         </is>
       </c>
-      <c r="FQ3" s="1" t="n"/>
       <c r="FR3" s="1" t="n"/>
       <c r="FS3" s="1" t="n"/>
       <c r="FT3" s="1" t="n"/>
-      <c r="FU3" s="21" t="inlineStr">
+      <c r="FU3" s="1" t="n"/>
+      <c r="FV3" s="21" t="inlineStr">
         <is>
           <t>Geluidsbelasting Geluidsbelasting belangrijke spoorwegen Lden 2021 (Exposition au bruit- aéroport)</t>
         </is>
       </c>
-      <c r="FV3" s="1" t="n"/>
       <c r="FW3" s="1" t="n"/>
       <c r="FX3" s="1" t="n"/>
       <c r="FY3" s="1" t="n"/>
-      <c r="FZ3" s="83" t="inlineStr">
+      <c r="FZ3" s="1" t="n"/>
+      <c r="GA3" s="83" t="inlineStr">
         <is>
           <t>Bodem is licht verontreinigd</t>
         </is>
       </c>
-      <c r="GA3" s="84" t="inlineStr">
+      <c r="GB3" s="84" t="inlineStr">
         <is>
           <t>Bodem is proper</t>
         </is>
       </c>
-      <c r="GB3" s="85" t="inlineStr">
+      <c r="GC3" s="85" t="inlineStr">
         <is>
           <t>Bodem is verontreinigd</t>
         </is>
       </c>
-      <c r="GC3" s="86" t="inlineStr">
+      <c r="GD3" s="86" t="inlineStr">
         <is>
           <t>Bodeminfo wordt gecheckt</t>
         </is>
       </c>
-      <c r="GD3" s="80" t="inlineStr">
+      <c r="GE3" s="80" t="inlineStr">
         <is>
           <t>Mogelijke risicogrond</t>
         </is>
       </c>
-      <c r="GE3" s="81" t="inlineStr">
+      <c r="GF3" s="81" t="inlineStr">
         <is>
           <t>Geen bodeminfo</t>
         </is>
       </c>
-      <c r="GF3" s="19" t="inlineStr">
+      <c r="GG3" s="19" t="inlineStr">
         <is>
           <t>Woningbouwgebieden</t>
         </is>
       </c>
-      <c r="GG3" s="78" t="inlineStr">
+      <c r="GH3" s="78" t="inlineStr">
         <is>
           <t>Woonvernieuwingsgebieden</t>
         </is>
@@ -3067,11 +3074,7 @@
         </is>
       </c>
       <c r="AE4" s="89" t="n"/>
-      <c r="AF4" s="89" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="AF4" s="89" t="n"/>
       <c r="AG4" s="89" t="inlineStr">
         <is>
           <t>/</t>
@@ -3457,91 +3460,91 @@
           <t>/</t>
         </is>
       </c>
-      <c r="DF4" s="105" t="inlineStr">
+      <c r="DF4" s="89" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="DG4" s="105" t="inlineStr">
         <is>
           <t>Geen overstroming gemodelleerd</t>
         </is>
       </c>
-      <c r="DG4" s="106" t="inlineStr">
+      <c r="DH4" s="106" t="inlineStr">
         <is>
           <t>Kleine kans op overstromingen onder klimaatverandering</t>
         </is>
       </c>
-      <c r="DH4" s="107" t="inlineStr">
+      <c r="DI4" s="107" t="inlineStr">
         <is>
           <t>Kleine kans op overstromingen</t>
         </is>
       </c>
-      <c r="DI4" s="108" t="inlineStr">
+      <c r="DJ4" s="108" t="inlineStr">
         <is>
           <t>Middelgrote kans op overstromingen</t>
         </is>
       </c>
-      <c r="DJ4" s="105" t="inlineStr">
+      <c r="DK4" s="105" t="inlineStr">
         <is>
           <t>Geen overstroming gemodelleerd</t>
         </is>
       </c>
-      <c r="DK4" s="106" t="inlineStr">
+      <c r="DL4" s="106" t="inlineStr">
         <is>
           <t>Kleine kans op overstromingen onder klimaatverandering</t>
         </is>
       </c>
-      <c r="DL4" s="107" t="inlineStr">
+      <c r="DM4" s="107" t="inlineStr">
         <is>
           <t>Kleine kans op overstromingen</t>
         </is>
       </c>
-      <c r="DM4" s="108" t="inlineStr">
+      <c r="DN4" s="108" t="inlineStr">
         <is>
           <t>Middelgrote kans op overstromingen</t>
         </is>
       </c>
-      <c r="DN4" s="105" t="inlineStr">
+      <c r="DO4" s="105" t="inlineStr">
         <is>
           <t>Geen overstroming gemodelleerd</t>
         </is>
       </c>
-      <c r="DO4" s="106" t="inlineStr">
+      <c r="DP4" s="106" t="inlineStr">
         <is>
           <t>Kleine kans op overstromingen onder klimaatverandering</t>
         </is>
       </c>
-      <c r="DP4" s="107" t="inlineStr">
+      <c r="DQ4" s="107" t="inlineStr">
         <is>
           <t>Kleine kans op overstromingen</t>
         </is>
       </c>
-      <c r="DQ4" s="108" t="inlineStr">
+      <c r="DR4" s="108" t="inlineStr">
         <is>
           <t>Middelgrote kans op overstromingen</t>
         </is>
       </c>
-      <c r="DR4" s="109" t="inlineStr">
+      <c r="DS4" s="109" t="inlineStr">
         <is>
           <t>IWB OeverzoneI</t>
         </is>
       </c>
-      <c r="DS4" s="109" t="inlineStr">
+      <c r="DT4" s="109" t="inlineStr">
         <is>
           <t>WB Overstromingsgebied</t>
         </is>
       </c>
-      <c r="DT4" s="110" t="inlineStr">
+      <c r="DU4" s="110" t="inlineStr">
         <is>
           <t>Bouwvrije opgave</t>
         </is>
       </c>
-      <c r="DU4" s="111" t="inlineStr">
+      <c r="DV4" s="111" t="inlineStr">
         <is>
           <t>Verscherpte watertoets</t>
         </is>
       </c>
-      <c r="DV4" s="89" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
       <c r="DW4" s="89" t="inlineStr">
         <is>
           <t>/</t>
@@ -3572,41 +3575,41 @@
           <t>/</t>
         </is>
       </c>
-      <c r="EC4" s="90" t="inlineStr">
+      <c r="EC4" s="89" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="ED4" s="90" t="inlineStr">
         <is>
           <t>0,5-5 ha</t>
         </is>
       </c>
-      <c r="ED4" s="91" t="inlineStr">
+      <c r="EE4" s="91" t="inlineStr">
         <is>
           <t>5-10 ha</t>
         </is>
       </c>
-      <c r="EE4" s="92" t="inlineStr">
+      <c r="EF4" s="92" t="inlineStr">
         <is>
           <t>10-20ha</t>
         </is>
       </c>
-      <c r="EF4" s="93" t="inlineStr">
+      <c r="EG4" s="93" t="inlineStr">
         <is>
           <t>20-50 ha</t>
         </is>
       </c>
-      <c r="EG4" s="94" t="inlineStr">
+      <c r="EH4" s="94" t="inlineStr">
         <is>
           <t>50-100 ha</t>
         </is>
       </c>
-      <c r="EH4" s="95" t="inlineStr">
+      <c r="EI4" s="95" t="inlineStr">
         <is>
           <t>&gt;100 ha</t>
         </is>
       </c>
-      <c r="EI4" s="89" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
       <c r="EJ4" s="89" t="inlineStr">
         <is>
           <t>/</t>
@@ -3742,86 +3745,86 @@
           <t>/</t>
         </is>
       </c>
-      <c r="FK4" s="96" t="inlineStr">
+      <c r="FK4" s="89" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="FL4" s="96" t="inlineStr">
         <is>
           <t>50-55 dB (décibel)</t>
         </is>
       </c>
-      <c r="FL4" s="97" t="inlineStr">
+      <c r="FM4" s="97" t="inlineStr">
         <is>
           <t>55-60 dB</t>
         </is>
       </c>
-      <c r="FM4" s="98" t="inlineStr">
+      <c r="FN4" s="98" t="inlineStr">
         <is>
           <t>60-65 dB</t>
         </is>
       </c>
-      <c r="FN4" s="99" t="inlineStr">
+      <c r="FO4" s="99" t="inlineStr">
         <is>
           <t>65-70 dB</t>
         </is>
       </c>
-      <c r="FO4" s="100" t="inlineStr">
+      <c r="FP4" s="100" t="inlineStr">
         <is>
           <t>&gt; 70 dB</t>
         </is>
       </c>
-      <c r="FP4" s="96" t="inlineStr">
+      <c r="FQ4" s="96" t="inlineStr">
         <is>
           <t>50-55 dB (décibel)</t>
         </is>
       </c>
-      <c r="FQ4" s="97" t="inlineStr">
+      <c r="FR4" s="97" t="inlineStr">
         <is>
           <t>55-60 dB</t>
         </is>
       </c>
-      <c r="FR4" s="98" t="inlineStr">
+      <c r="FS4" s="98" t="inlineStr">
         <is>
           <t>60-65 dB</t>
         </is>
       </c>
-      <c r="FS4" s="99" t="inlineStr">
+      <c r="FT4" s="99" t="inlineStr">
         <is>
           <t>65-70 dB</t>
         </is>
       </c>
-      <c r="FT4" s="100" t="inlineStr">
+      <c r="FU4" s="100" t="inlineStr">
         <is>
           <t>&gt; 70 dB</t>
         </is>
       </c>
-      <c r="FU4" s="96" t="inlineStr">
+      <c r="FV4" s="96" t="inlineStr">
         <is>
           <t>50-55 dB (décibel)</t>
         </is>
       </c>
-      <c r="FV4" s="97" t="inlineStr">
+      <c r="FW4" s="97" t="inlineStr">
         <is>
           <t>55-60 dB</t>
         </is>
       </c>
-      <c r="FW4" s="98" t="inlineStr">
+      <c r="FX4" s="98" t="inlineStr">
         <is>
           <t>60-65 dB</t>
         </is>
       </c>
-      <c r="FX4" s="99" t="inlineStr">
+      <c r="FY4" s="99" t="inlineStr">
         <is>
           <t>65-70 dB</t>
         </is>
       </c>
-      <c r="FY4" s="100" t="inlineStr">
+      <c r="FZ4" s="100" t="inlineStr">
         <is>
           <t>&gt; 70 dB</t>
         </is>
       </c>
-      <c r="FZ4" s="101" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
       <c r="GA4" s="101" t="inlineStr">
         <is>
           <t>/</t>
@@ -3837,12 +3840,17 @@
           <t>/</t>
         </is>
       </c>
-      <c r="GF4" s="101" t="inlineStr">
+      <c r="GD4" s="101" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
       <c r="GG4" s="101" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="GH4" s="101" t="inlineStr">
         <is>
           <t>/</t>
         </is>
@@ -3850,12 +3858,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="DN3:DQ3"/>
-    <mergeCell ref="DF2:DQ2"/>
-    <mergeCell ref="DT3:DU3"/>
-    <mergeCell ref="DR3:DS3"/>
-    <mergeCell ref="DF3:DI3"/>
-    <mergeCell ref="DJ3:DM3"/>
+    <mergeCell ref="DK3:DN3"/>
+    <mergeCell ref="DO3:DR3"/>
+    <mergeCell ref="DU3:DV3"/>
+    <mergeCell ref="DG2:DR2"/>
+    <mergeCell ref="DS3:DT3"/>
+    <mergeCell ref="DG3:DJ3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>